<commit_message>
Compeed manual overrides materialized
</commit_message>
<xml_diff>
--- a/seasonal-catalog.xlsx
+++ b/seasonal-catalog.xlsx
@@ -4137,7 +4137,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Επιθέματα για Σπυράκια* Conceal &amp; Go | Compeed®</t>
+          <t xml:space="preserve">Compeed Επιθέματα για Φουσκάλες στο Πέλμα από Αθλητικές Δραστηριότητες x5</t>
         </is>
       </c>
       <c r="B79">
@@ -4145,7 +4145,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Καθαρίστε, καλύψτε και προστατέψτε τα σπυράκια σας με τα Επιθέματα Compeed Conceal &amp; Go. Ανακαλύψτε πως η υδροκολλοειδή τεχνολογία των επιθεμάτων για σπυράκια βοηθάει στην αντιμετώπιση των σπυριών.</t>
+          <t xml:space="preserve">Τα Επιθέματα για Φουσκάλες στο Πέλμα από Αθλητικές Δραστηριότητες COMPEED® είναι ειδικά σχεδιασμένα ώστε να εφαρμόζουν στο μετατάρσιο (το μπροστινό τμήμα του πέλματος) και να παρέχουν προστασία από την τριβή</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4185,14 +4185,14 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t xml:space="preserve">www.compeed.gr</t>
+          <t xml:space="preserve">compeed.gr</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eeltplekkenpleisters Medium | Compeed®</t>
+          <t xml:space="preserve">Compeed Μεσαία Επιθέματα για Φουσκάλες x5</t>
         </is>
       </c>
       <c r="B80">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPEED® Eeltplekkenpleisters Medium beschermt tegen wrijving door als een tweede huid te werken. Wacht niet langer om de pijn te verlichten en eelt te elimineren.</t>
+          <t xml:space="preserve">Τα Μεσαία Επιθέματα για Φουσκάλες COMPEED® απορροφούν την περιττή υγρασία και σχηματίζουν ένα προστατευτικό μαξιλάρι προσφέροντας άμεση ανακούφιση από τον πόνο και ιδανικές συνθήκες για την επούλωση των φουσκαλών του ποδιού.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4247,7 +4247,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Επιθέματα για Σπυράκια* Καθαρισμού | Compeed ®</t>
+          <t xml:space="preserve">Compeed Επιθέματα για Φουσκάλες στα Δάκτυλα των Ποδιών x8</t>
         </is>
       </c>
       <c r="B81">
@@ -4255,7 +4255,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Καθαρίστε, ενυδατώστε και φωτίστε το δέρμα σας με τα Επιθέματα για Σπυράκια* COMPEED® Καθαρισμού. Μάθετε πώς τα υδροκολλοειδή επιθέματα για τα σπυράκια βοηθούν στην απομάκρυνση των ακαθαρσιών του δέρματος.</t>
+          <t xml:space="preserve">Τα επιθέματα για φουσκάλες στα δάκτυλα των ποδιών COMPEED® είναι ειδικά σχεδιασμένα για φουσκάλες που εμφανίζονται στα δάκτυλα των ποδιών, συχνά σε δυσπρόσιτα σημεία, και παρέχουν άμεση ανακούφιση από τον πόνο.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4295,14 +4295,14 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t xml:space="preserve">www.compeed.gr</t>
+          <t xml:space="preserve">compeed.gr</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPEED® Advanced Corn Care</t>
+          <t xml:space="preserve">Compeed Μεσαία Επιθέματα για Κάλους στα Μικρά Δάκτυλα των Ποδιών x10</t>
         </is>
       </c>
       <c r="B82">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPEED® Corn cuhions contain hydrocolloid active gel technology which relieves pain immediately and helps remove the corn</t>
+          <t xml:space="preserve">Τα Επιθέματα για Κάλους στα Δάκτυλα των Ποδιών COMPEED® περιέχουν ενεργή γέλη υδροκολλοειδούς τεχνολογίας η οποία καταπραΰνει αμέσως τον πόνο και βοηθά στην αφαίρεση της σκλήρυνσης</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4357,7 +4357,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blarenpleisters Small | Compeed® | Behandeling van kleine blaren</t>
+          <t xml:space="preserve">Compeed Μικρά Επιθέματα για Φουσκάλες x6</t>
         </is>
       </c>
       <c r="B83">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPEED® Blarenpleisters Small is speciaal ontworpen voor de niet-vlakke zijvlakken van uw voet en voor kleine blaren</t>
+          <t xml:space="preserve">Τα Μικρά Επιθέματα για Φουσκάλες COMPEED® απορροφούν την περιττή υγρασία και σχηματίζουν ένα προστατευτικό μαξιλάρι προσφέροντας άμεση ανακούφιση από τον πόνο και ιδανικές συνθήκες για την επούλωση των φουσκαλών του ποδιού</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4412,7 +4412,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Επιθέματα για Σπυράκια* Conceal &amp; Go | Compeed®</t>
+          <t xml:space="preserve">Compeed Επιθέματα για Κότσι x5</t>
         </is>
       </c>
       <c r="B84">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Καθαρίστε, καλύψτε και προστατέψτε τα σπυράκια σας με τα Επιθέματα Compeed Conceal &amp; Go. Ανακαλύψτε πως η υδροκολλοειδή τεχνολογία των επιθεμάτων για σπυράκια βοηθάει στην αντιμετώπιση των σπυριών.</t>
+          <t xml:space="preserve">Τα Επιθέματα για Κότσι COMPEED® βοηθούν στην πρόληψη της δημιουργίας φουσκαλών και της περαιτέρω σκλήρυνσης του δέρματος η οποία μπορεί να προκαλέσει άλλες επώδυνες δερματικές καταστάσεις</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4460,14 +4460,14 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t xml:space="preserve">www.compeed.gr</t>
+          <t xml:space="preserve">compeed.gr</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Επιθέματα για Σπυράκια* Conceal &amp; Go | Compeed®</t>
+          <t xml:space="preserve">Compeed Μεγάλα Επιθέματα για Σκληρύνσεις x2</t>
         </is>
       </c>
       <c r="B85">
@@ -4475,7 +4475,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Καθαρίστε, καλύψτε και προστατέψτε τα σπυράκια σας με τα Επιθέματα Compeed Conceal &amp; Go. Ανακαλύψτε πως η υδροκολλοειδή τεχνολογία των επιθεμάτων για σπυράκια βοηθάει στην αντιμετώπιση των σπυριών.</t>
+          <t xml:space="preserve">Τα Επιθέματα για Σκληρύνσεις COMPEED® περιέχουν ενεργή γέλη υδροκολλοειδούς τεχνολογίας η οποία καταπραΰνει αμέσως τον πόνο και βοηθά στην αφαίρεση των σκληρύνσεων.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4515,14 +4515,14 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t xml:space="preserve">www.compeed.gr</t>
+          <t xml:space="preserve">compeed.gr</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Επιθέματα για Σπυράκια* Καθαρισμού | Compeed ®</t>
+          <t xml:space="preserve">Compeed Μεσαία Επιθέματα για Σκληρύνσεις x6</t>
         </is>
       </c>
       <c r="B86">
@@ -4530,7 +4530,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Καθαρίστε, ενυδατώστε και φωτίστε το δέρμα σας με τα Επιθέματα για Σπυράκια* COMPEED® Καθαρισμού. Μάθετε πώς τα υδροκολλοειδή επιθέματα για τα σπυράκια βοηθούν στην απομάκρυνση των ακαθαρσιών του δέρματος.</t>
+          <t xml:space="preserve">Τα Επιθέματα για Σκληρύνσεις COMPEED® περιέχουν ενεργή γέλη υδροκολλοειδούς τεχνολογίας η οποία καταπραΰνει αμέσως τον πόνο και βοηθά στην αφαίρεση των σκληρύνσεων.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4570,14 +4570,14 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t xml:space="preserve">www.compeed.gr</t>
+          <t xml:space="preserve">compeed.gr</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Επιθέματα για Σπυράκια* Καθαρισμού | Compeed ®</t>
+          <t xml:space="preserve">Compeed Μεσαία Επιθέματα για Κάλους Μεταξύ Δακτύλων x10</t>
         </is>
       </c>
       <c r="B87">
@@ -4585,7 +4585,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Καθαρίστε, ενυδατώστε και φωτίστε το δέρμα σας με τα Επιθέματα για Σπυράκια* COMPEED® Καθαρισμού. Μάθετε πώς τα υδροκολλοειδή επιθέματα για τα σπυράκια βοηθούν στην απομάκρυνση των ακαθαρσιών του δέρματος.</t>
+          <t xml:space="preserve">Τα Επιθέματα για Κάλους στα Δάκτυλα των Ποδιών COMPEED® περιέχουν ενεργή γέλη υδροκολλοειδούς τεχνολογίας η οποία καταπραΰνει αμέσως τον πόνο και βοηθά στην αφαίρεση της σκλήρυνσης</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4625,14 +4625,14 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t xml:space="preserve">www.compeed.gr</t>
+          <t xml:space="preserve">compeed.gr</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compeed® Anti-Imperfection* Patch Discreet, ideaal voor overdag</t>
+          <t xml:space="preserve">Compeed Αόρατο Επίθεμα για τον Επιχείλιο Έρπη x15</t>
         </is>
       </c>
       <c r="B88">
@@ -4640,7 +4640,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t xml:space="preserve">De discrete patch Compeed® Anti-Imperfection heeft 3-voudige werking: reinigen, verbergen en beschermen van kleine puistjes en zwarte puntjes</t>
+          <t xml:space="preserve">COMPEEDÂ® Discreet Cold sore patch contains hydrocolloid active gel technology for faster healing and scabbing prevention</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4687,7 +4687,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eeltplekkenpleisters Medium | Compeed®</t>
+          <t xml:space="preserve">Compeed Extreme Μεσαία Επιθέματα για Φουσκάλες x5</t>
         </is>
       </c>
       <c r="B89">
@@ -4695,7 +4695,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPEED® Eeltplekkenpleisters Medium beschermt tegen wrijving door als een tweede huid te werken. Wacht niet langer om de pijn te verlichten en eelt te elimineren.</t>
+          <t xml:space="preserve">Τα Μεσαία Επιθέματα για Φουσκάλες COMPEED® απορροφούν την περιττή υγρασία και σχηματίζουν ένα προστατευτικό μαξιλάρι προσφέροντας άμεση ανακούφιση από τον πόνο και ιδανικές συνθήκες για την επούλωση των φουσκαλών του ποδιού.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4742,7 +4742,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compeed® Anti-Imperfection* Patch Discreet, ideaal voor overdag</t>
+          <t xml:space="preserve">Compeed Επιθέματα για Σπυράκια Conceal &amp; Go x15</t>
         </is>
       </c>
       <c r="B90">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t xml:space="preserve">De discrete patch Compeed® Anti-Imperfection heeft 3-voudige werking: reinigen, verbergen en beschermen van kleine puistjes en zwarte puntjes</t>
+          <t xml:space="preserve">Καθαρίστε, καλύψτε και προστατέψτε τα σπυράκια σας με τα Επιθέματα Compeed Conceal &amp; Go. Ανακαλύψτε πως η υδροκολλοειδή τεχνολογία των επιθεμάτων για σπυράκια βοηθάει στην αντιμετώπιση των σπυριών.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4797,7 +4797,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compeed Plaster Stop Spots x7</t>
+          <t xml:space="preserve">Compeed Επιθέματα για Σπυράκια Καθαρισμού x7</t>
         </is>
       </c>
       <c r="B91">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εποχιακό προϊόν για προστασία ή ανακούφιση κατά τις θερινές δραστηριότητες. Προϊόν της σειράς Compeed (Stop Spots).</t>
+          <t xml:space="preserve">Καθαρίστε, ενυδατώστε και φωτίστε το δέρμα σας με τα Επιθέματα για Σπυράκια* COMPEED® Καθαρισμού. Μάθετε πώς τα υδροκολλοειδή επιθέματα για τα σπυράκια βοηθούν στην απομάκρυνση των ακαθαρσιών του δέρματος.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4841,13 +4841,18 @@
       <c r="J91" t="inlineStr">
         <is>
           <t xml:space="preserve">COMPEED PLASTER STOP SPOTS X7</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">compeed.gr</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eeltplekkenpleisters Medium | Compeed®</t>
+          <t xml:space="preserve">Compeed Μεσαία Ενυδατικά Επιθέματα για Κάλους x6</t>
         </is>
       </c>
       <c r="B92">
@@ -4855,7 +4860,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPEED® Eeltplekkenpleisters Medium beschermt tegen wrijving door als een tweede huid te werken. Wacht niet langer om de pijn te verlichten en eelt te elimineren.</t>
+          <t xml:space="preserve">Τα Ενυδατικά Επιθέματα για Κάλους COMPEED® μένουν σταθερά στη θέση τους για μέρες παρέχοντας προστασία από την τριβή και την πίεση</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -4902,7 +4907,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eeltplekkenpleisters Medium | Compeed®</t>
+          <t xml:space="preserve">Compeed Μεσαία Επιθέματα για Φουσκάλες x10</t>
         </is>
       </c>
       <c r="B93">
@@ -4910,7 +4915,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">COMPEED® Eeltplekkenpleisters Medium beschermt tegen wrijving door als een tweede huid te werken. Wacht niet langer om de pijn te verlichten en eelt te elimineren.</t>
+          <t xml:space="preserve">Τα Μεσαία Επιθέματα για Φουσκάλες COMPEED® απορροφούν την περιττή υγρασία και σχηματίζουν ένα προστατευτικό μαξιλάρι προσφέροντας άμεση ανακούφιση από τον πόνο και ιδανικές συνθήκες για την επούλωση των φουσκαλών του ποδιού.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -4957,7 +4962,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Επιθέματα για Σπυράκια* Conceal &amp; Go | Compeed®</t>
+          <t xml:space="preserve">Compeed Επιθέματα για Φουσκάλες από Ψηλοτάκουνα Παπούτσια x5</t>
         </is>
       </c>
       <c r="B94">
@@ -4965,7 +4970,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Καθαρίστε, καλύψτε και προστατέψτε τα σπυράκια σας με τα Επιθέματα Compeed Conceal &amp; Go. Ανακαλύψτε πως η υδροκολλοειδή τεχνολογία των επιθεμάτων για σπυράκια βοηθάει στην αντιμετώπιση των σπυριών.</t>
+          <t xml:space="preserve">Τα Επιθέματα για Φουσκάλες από Ψηλοτάκουνα Παπούτσια COMPEED® είναι κατάλληλα για όλες τις φουσκάλες που προκαλούνται από ψηλοτάκουνα παπούτσια</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5005,14 +5010,14 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t xml:space="preserve">www.compeed.gr</t>
+          <t xml:space="preserve">compeed.gr</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pansement Ampoules Assortiment - Pack 3 en 1 | Compeed®</t>
+          <t xml:space="preserve">Compeed Επιθέματα Διαφορετικών Μεγεθών για Φουσκάλες x5</t>
         </is>
       </c>
       <c r="B95">
@@ -5020,7 +5025,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Le pansement COMPEED® Ampoules Assortiment est la solution pratique pour soigner tous les types d’ampoules au pied grâce à ses 3 formats différents.</t>
+          <t xml:space="preserve">Η συσκευασία Επιθέματα Διαφορετικών Μεγεθών για Φουσκάλες COMPEED® περιλαμβάνει 2 Μεσαία Επιθέματα για Φουσκάλες, 2 Μικρά Επιθέματα για Φουσκάλες και 1 Επίθεμα για Φουσκάλες στα Δάκτυλα των Ποδιών. Ιδανική για κιτ πρώτων βοηθειών!</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">

</xml_diff>

<commit_message>
CER-8 overrides + local Vican images (203 synced)
</commit_message>
<xml_diff>
--- a/seasonal-catalog.xlsx
+++ b/seasonal-catalog.xlsx
@@ -743,11 +743,6 @@
           <t xml:space="preserve">Superfood Slim Detox</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">seasonal/superfood-slim-detox-liquid-300ml-5213006870002.png</t>
-        </is>
-      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t xml:space="preserve">2200032078</t>
@@ -1827,7 +1822,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">CER-8 Παιδικό Εντομοαπωθητικό Strips x24</t>
+          <t xml:space="preserve">CER-8 Microcapsules Patch Junior x24</t>
         </is>
       </c>
       <c r="B34">
@@ -1835,7 +1830,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εποχιακό προϊόν για προστασία ή ανακούφιση κατά τις θερινές δραστηριότητες. Προϊόν της σειράς CER-8 (Kids).</t>
+          <t xml:space="preserve">Παιδικά εντομοαπωθητικά αυτοκόλλητα με καινοτομία μικροκάψουλας που απαλλάσσουν από τα ενοχλητικά τσιμπήματα των κουνουπιών, δημιουργώντας μια ακτίνα προστασίας ενός μέτρου (1m) έως και έξι ώρες. Μπορεί να κολληθεί σε ρούχα, έπιπλα, ακόμη και στην κούνια του μωρού σε σημείο μη ορατό και προσβάσιμο από τα παιδιά. Το πρωτοποριακό αυτό αυτοκόλλητο περιέχει μικροκάψουλες με το δραστικό συστατικό Εucalyptus Citriodora oil, το οποίο προστατεύει αποτελεσματικά απο τα κουνούπια και τις σκνίπες, συμπεριλαμβανομένου του ασιατικού κουνουπιού</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1855,7 +1850,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/cer-8-strips-x24-5204559030012.jpg</t>
+          <t xml:space="preserve">vican/cer-8-microcapsules-patch-junior-5204559030012.jpg</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1871,13 +1866,18 @@
       <c r="J34" t="inlineStr">
         <is>
           <t xml:space="preserve">CER 8 ΠΑΙΔ.ΕΝΤΟΜΟΑΠ.STRIPS X24STR</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vican.gr</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">CER-8 Anti-Mosquito Spray Άοσμο 100ml</t>
+          <t xml:space="preserve">CER-8 Άοσμο Εντομοαπωθητικό Spray 100ml</t>
         </is>
       </c>
       <c r="B35">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εποχιακό προϊόν για προστασία ή ανακούφιση κατά τις θερινές δραστηριότητες. Προϊόν της σειράς CER-8 (Anti-Mosquito).</t>
+          <t xml:space="preserve">Το άοσμο εντομοαπωθητικό Cer’8 προστατεύει αποτελεσματικά από τα κουνούπια και τις σκνίπες, συμπεριλαμβανομένου του ασιατικού κουνουπιού</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/cer-8-anti-mosquito-spray-100ml-5204559030319.jpg</t>
+          <t xml:space="preserve">vican/cer-8-5204559030319.jpg</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1921,6 +1921,11 @@
       <c r="J35" t="inlineStr">
         <is>
           <t xml:space="preserve">CER-8 ANTI-MOSQ.SPRAY ΑΟΣΜΟ 100ML</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vican.gr</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1940,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εποχιακό προϊόν για προστασία ή ανακούφιση κατά τις θερινές δραστηριότητες. Προϊόν της σειράς CER-8 (Lotion).</t>
+          <t xml:space="preserve">Η εντομοαπωθητική lotion Cer’8 χαρίζει προστασία σε όλη την οικογένεια. Χάρη στη σύνθεσή της με Eucalyptus Citriodora Oil, προφυλάσσει αποτελεσματικά έως πέντε ώρες από τα κουνούπια και τις σκνίπες, συμπεριλαμβανομένου του ασιατικού κουνουπιού</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1955,7 +1960,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/cer-8-lotion-125ml-5204559030074.jpg</t>
+          <t xml:space="preserve">vican/cer-8-lotion-5204559030074.jpg</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1971,13 +1976,18 @@
       <c r="J36" t="inlineStr">
         <is>
           <t xml:space="preserve">CER-8 ΕΝΤΟΜΟΑΠΩΘ. LOTION 125ML</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vican.gr</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">CER-8 Εντομοαπωθητικά Strips x24</t>
+          <t xml:space="preserve">CER-8 Microcapsules Patch Ενηλίκων x24</t>
         </is>
       </c>
       <c r="B37">
@@ -1985,7 +1995,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εποχιακό προϊόν για προστασία ή ανακούφιση κατά τις θερινές δραστηριότητες. Προϊόν της σειράς CER-8 (Strips).</t>
+          <t xml:space="preserve">Εντομοαπωθητικά αυτοκόλλητα ενηλίκων με καινοτομία μικροκάψουλας που απαλλάσσουν από τα ενοχλητικά τσιμπήματα των κουνουπιών, δημιουργώντας μια ακτίνα προστασίας ενός μέτρου (1m) έως και έξι ώρες. Μπορεί να κολληθεί στο κρεβάτι, στα ρούχα ή άλλα αντικείμενα. Με το δραστικό συστατικό Eucalyptus Citriodora oil, το οποίο προστατεύει αποτελεσματικά απο τα κουνούπια και τις σκνίπες, συμπεριλαμβανομένου του ασιατικού κουνουπιού</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2005,7 +2015,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/cer-8-strips-x24-5204559030005.jpg</t>
+          <t xml:space="preserve">vican/cer-8-microcapsules-patch-5204559030005.jpg</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2021,13 +2031,18 @@
       <c r="J37" t="inlineStr">
         <is>
           <t xml:space="preserve">CER-8 ΕΝΤΟΜΟΑΠΩΘ. STRIPS X24 STRI</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vican.gr</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">CER-8 Ultra Protect Spray Άοσμο 30ml</t>
+          <t xml:space="preserve">CER-8 Mini Άοσμο Εντομοαπωθητικό Spray 30ml</t>
         </is>
       </c>
       <c r="B38">
@@ -2035,7 +2050,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εποχιακό προϊόν για προστασία ή ανακούφιση κατά τις θερινές δραστηριότητες. Προϊόν της σειράς CER-8 (Ultra Protect).</t>
+          <t xml:space="preserve">Το άοσμο εντομοαπωθητικό Cer’8 προστατεύει αποτελεσματικά από τα κουνούπια και τις σκνίπες, συμπεριλαμβανομένου του ασιατικού κουνουπιού</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2055,7 +2070,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/cer-8-ultra-protect-spray-30ml-5204559030166.jpg</t>
+          <t xml:space="preserve">vican/cer-8-mini-spray-5204559030166.jpg</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2071,6 +2086,11 @@
       <c r="J38" t="inlineStr">
         <is>
           <t xml:space="preserve">CER-8 ULTRA PROTECT.SPR.ΑΟΣΜ.MIN30</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vican.gr</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2197,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">CER-8 Patch Junior Microcaps Εντομοαπωθητικά x48</t>
+          <t xml:space="preserve">CER-8 Microcapsules Patch Junior Economy Pack x48</t>
         </is>
       </c>
       <c r="B41">
@@ -2185,7 +2205,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εποχιακό προϊόν για προστασία ή ανακούφιση κατά τις θερινές δραστηριότητες. Προϊόν της σειράς CER-8 (Junior).</t>
+          <t xml:space="preserve">Παιδικά εντομοαπωθητικά αυτοκόλλητα με καινοτομία μικροκάψουλας που απαλλάσσουν από τα ενοχλητικά τσιμπήματα των κουνουπιών, δημιουργώντας μια ακτίνα προστασίας ενός μέτρου (1m) έως και έξι ώρες. Μπορεί να κολληθεί σε ρούχα, έπιπλα, ακόμη και στην κούνια του μωρού σε σημείο μη ορατό και προσβάσιμο από τα παιδιά. Με το δραστικό συστατικό Εucalyptus Citriodora oil, το οποίο προστατεύει αποτελεσματικά απο τα κουνούπι και τις σκνίπες, συμπεριλαμβανομένου του ασιατικού κουνουπιού</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2205,7 +2225,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/cer-8-patch-junior-microcaps-x48-5204559030111.jpg</t>
+          <t xml:space="preserve">vican/cer-8-microcapsules-patch-junior-economy-pack-5204559030111.jpg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2221,13 +2241,18 @@
       <c r="J41" t="inlineStr">
         <is>
           <t xml:space="preserve">CER-8 PATCH JUNIOR MICROC.ΕΝΤΟ/ΚΟ48</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vican.gr</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">CER-8 Roll-On After Bite 10ml</t>
+          <t xml:space="preserve">CER-8 After Bite Roll-On 10ml</t>
         </is>
       </c>
       <c r="B42">
@@ -2235,7 +2260,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εποχιακό προϊόν για προστασία ή ανακούφιση κατά τις θερινές δραστηριότητες. Προϊόν της σειράς CER-8 (After Bite).</t>
+          <t xml:space="preserve">Η πιο φυσική και αποτελεσματική λύση ανακούφισης από τα τσιμπήματα των κουνουπιών. Με συστατικά γνωστά για τις αντιφλογιστικές και αντι-ερεθιστικές τους ιδιότητες (Πρόπολη, Χαμομήλι, Καλέντουλα, Αλόη), ανακουφίζει άμεσα από τα ενοχλητικά συμπτώματα του τσιμπήματος, όπως ερεθισμός, αίσθημα κνησμού, ερύθυμα. Με Πρόπολη, Αλόη, Φασκόμηλο, Χαμομήλι, Καλέντουλα, Πολυδοκανόλη.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2255,7 +2280,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/cer-8-roll-on-after-bite-10ml-5204559030043.jpg</t>
+          <t xml:space="preserve">vican/cer-8-5204559030043.jpg</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2271,13 +2296,18 @@
       <c r="J42" t="inlineStr">
         <is>
           <t xml:space="preserve">CER-8 ROLL-ON AFTER BITE 10ML</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vican.gr</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">CER-8 Stickers After Bite x30</t>
+          <t xml:space="preserve">CER-8 After Bite Stickers x30</t>
         </is>
       </c>
       <c r="B43">
@@ -2285,7 +2315,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Εποχιακό προϊόν για προστασία ή ανακούφιση κατά τις θερινές δραστηριότητες. Προϊόν της σειράς CER-8 (After Bite).</t>
+          <t xml:space="preserve">Τα παιδικά επιθέματα Cer’8 After Bite Stickers συμβάλλουν στην άμεση καταπράυνση από τα τσιμπήματα των εντόμων, χάρη στη φυτική τους σύνθεση από Καλέντουλα, Βιταμίνη Ε και Έλαιο σταφυλιού. Ανακουφίζουν από το αίσθημα του κνησμού και βοηθούν στη μείωση του οιδήματος και του ερεθισμού. Έχουν απίθανα σχέδια και αποτρέπουν τα παιδιά από το να ξύσουν την κνησμώδη περιοχή του τσιμπήματος. Ιδανικά και για</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2305,7 +2335,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/cer-8-stickers-after-bite-x30-5204559030098.jpg</t>
+          <t xml:space="preserve">vican/cer-8-after-bite-stickers-5204559030098.jpg</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2321,6 +2351,11 @@
       <c r="J43" t="inlineStr">
         <is>
           <t xml:space="preserve">CER-8 STICKERS AFTER BITE X30</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vican.gr</t>
         </is>
       </c>
     </row>
@@ -4165,7 +4200,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-underfoot-x5-3574660559859.jpg</t>
+          <t xml:space="preserve">seasonal/x5-3574660559859.png</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -4220,7 +4255,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-medium-x5-3663555001457.jpg</t>
+          <t xml:space="preserve">seasonal/x5-3663555001457.png</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4275,7 +4310,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-x8-3663555001679.jpg</t>
+          <t xml:space="preserve">seasonal/x8-3663555001679.png</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -4330,7 +4365,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-medium-corn-x10-3663555001969.jpg</t>
+          <t xml:space="preserve">seasonal/x10-3663555001969.png</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -4385,7 +4420,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-small-x6-3663555001440.webp</t>
+          <t xml:space="preserve">seasonal/x6-3663555001440.png</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -4440,7 +4475,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-x5-3663555001938.png</t>
+          <t xml:space="preserve">seasonal/x5-3663555001938.png</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4495,7 +4530,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-large-x2-3663555001549.jpg</t>
+          <t xml:space="preserve">seasonal/x2-3663555001549.png</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4550,7 +4585,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-medium-x6-3663555001945.jpg</t>
+          <t xml:space="preserve">seasonal/x6-3663555001945.png</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4605,7 +4640,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-medium-x10-3663555001952.jpg</t>
+          <t xml:space="preserve">seasonal/x10-3663555001952.png</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4660,7 +4695,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-patch-x15-3663555002126.jpg</t>
+          <t xml:space="preserve">seasonal/x15-3663555002126.png</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4715,7 +4750,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-extreme-medium-x5-3663555002386.jpg</t>
+          <t xml:space="preserve">seasonal/extreme-x5-3663555002386.png</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -4770,7 +4805,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-patch-stop-spots-x15-3663555005394.png</t>
+          <t xml:space="preserve">seasonal/conceal-go-x15-3663555005394.png</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -4825,7 +4860,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-plaster-stop-spots-x7-3663555005349.jpg</t>
+          <t xml:space="preserve">seasonal/x7-3663555005349.png</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4880,7 +4915,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-medium-moisturizing-corn-x6-3663555002492.png</t>
+          <t xml:space="preserve">seasonal/x6-3663555002492.png</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4935,7 +4970,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-medium-x10-3663555002973.jpg</t>
+          <t xml:space="preserve">seasonal/x10-3663555002973.png</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4990,7 +5025,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-x5-3663555002652.webp</t>
+          <t xml:space="preserve">seasonal/x5-3663555002652.png</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -5045,7 +5080,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t xml:space="preserve">seasonal/compeed-mix-pack-5-x-3-3663555002744.png</t>
+          <t xml:space="preserve">seasonal/x5-3663555002744.png</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">

</xml_diff>